<commit_message>
Consolidate demo to one workbook per framework; add AC-17 multi-tenant control
- Add AC-17 (Remote Access) as the 8th control in the 800-53 demo workbook,
  left unassessed so it flows to the assessor. Diverges across the two demo
  CRMs — AWS GovCloud = Customer (customer-configured VPN/conditional access),
  Azure Government = Inherited (managed Azure Bastion) — so attaching both CRMs
  produces a genuinely different per-scope verdict/narrative per tenant.
- Fix SC-7 demo row: an inherited control is Compliant (applicable, met by the
  provider), not Not Applicable. Inherited=Compliant, N/A=N/A are distinct.
- Delete the duplicate demo/ccis/ workbook + its builder (_build_demo_ccis.py)
  and _verify_ccis_coverage.py. One demo workbook per framework now lives in
  demo/workbooks/ as intended.
- Update demo/README.md + EVIDENCE_CHAIN_DEMO.md to point at
  demo/workbooks/DEMO_NIST_800-53r5 and reflect the 8-control set.
</commit_message>
<xml_diff>
--- a/demo/crm/AWS_GovCloud_FedRAMP_High_CRM.xlsx
+++ b/demo/crm/AWS_GovCloud_FedRAMP_High_CRM.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1915,12 +1915,12 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>AT-1</t>
+          <t>AC-17</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Awareness and Training Policy and Procedures</t>
+          <t>Remote Access</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -1930,12 +1930,12 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Not applicable to the AWS service boundary. Customer maintains the customer-side awareness and training policy independently.</t>
+          <t>AWS provides the network primitives (Client VPN, Verified Access, Security Groups, IAM) but does not configure or operate the customer's remote-access policy or endpoints.</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Customer is responsible for developing, documenting, disseminating, reviewing, and updating the customer security awareness and training policy and supporting procedures applicable to all customer personnel with access to customer information systems.</t>
+          <t>Customer is responsible for authorizing remote access prior to connection and enforcing approved methods: AWS Client VPN with certificate + IdP authentication, conditional-access rules, session logging to CloudWatch, and periodic review of remote-access entitlements.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -1947,12 +1947,12 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>AT-2</t>
+          <t>AT-1</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Literacy Training and Awareness</t>
+          <t>Awareness and Training Policy and Procedures</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -1962,12 +1962,12 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Not applicable to the AWS service boundary.</t>
+          <t>Not applicable to the AWS service boundary. Customer maintains the customer-side awareness and training policy independently.</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Customer is responsible for providing security literacy training and awareness to all customer information system users on initial access, annually thereafter, and following any significant change to the system environment, including role-based content per the customer training program.</t>
+          <t>Customer is responsible for developing, documenting, disseminating, reviewing, and updating the customer security awareness and training policy and supporting procedures applicable to all customer personnel with access to customer information systems.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -1979,12 +1979,12 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>AT-3</t>
+          <t>AT-2</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Role-Based Training</t>
+          <t>Literacy Training and Awareness</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -1999,7 +1999,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Customer is responsible for providing role-based security training to customer personnel with significant security responsibilities (cloud administrators, security engineers, developers with production access) prior to authorizing access and annually thereafter.</t>
+          <t>Customer is responsible for providing security literacy training and awareness to all customer information system users on initial access, annually thereafter, and following any significant change to the system environment, including role-based content per the customer training program.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2011,12 +2011,12 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>PL-2</t>
+          <t>AT-3</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>System Security and Privacy Plans</t>
+          <t>Role-Based Training</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2026,12 +2026,12 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Not applicable to the AWS service boundary. Customer maintains the customer-side System Security Plan independently.</t>
+          <t>Not applicable to the AWS service boundary.</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Customer is responsible for developing, documenting, and maintaining the customer System Security Plan covering customer-deployed workloads, customer responsibilities, and the explicit inheritance and shared responsibility relationships with AWS per this CRM.</t>
+          <t>Customer is responsible for providing role-based security training to customer personnel with significant security responsibilities (cloud administrators, security engineers, developers with production access) prior to authorizing access and annually thereafter.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -2043,12 +2043,12 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>PL-4</t>
+          <t>PL-2</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Rules of Behavior</t>
+          <t>System Security and Privacy Plans</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -2058,12 +2058,12 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Not applicable to the AWS service boundary.</t>
+          <t>Not applicable to the AWS service boundary. Customer maintains the customer-side System Security Plan independently.</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Customer is responsible for establishing and enforcing rules of behavior for customer users with access to customer-managed AWS resources, including acknowledgment prior to access authorization.</t>
+          <t>Customer is responsible for developing, documenting, and maintaining the customer System Security Plan covering customer-deployed workloads, customer responsibilities, and the explicit inheritance and shared responsibility relationships with AWS per this CRM.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -2075,12 +2075,12 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>PM-1</t>
+          <t>PL-4</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Information Security Program Plan</t>
+          <t>Rules of Behavior</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2095,7 +2095,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Customer is responsible for establishing and maintaining the customer Information Security Program Plan, including customer governance, risk, compliance functions, and senior agency information security officer designation.</t>
+          <t>Customer is responsible for establishing and enforcing rules of behavior for customer users with access to customer-managed AWS resources, including acknowledgment prior to access authorization.</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -2107,12 +2107,12 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>PM-9</t>
+          <t>PM-1</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Risk Management Strategy</t>
+          <t>Information Security Program Plan</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -2127,7 +2127,7 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Customer is responsible for developing and implementing the customer Risk Management Strategy, including risk tolerance levels for customer-managed workloads in AWS GovCloud and risk framing for the inherited and shared portions of the AWS shared responsibility model.</t>
+          <t>Customer is responsible for establishing and maintaining the customer Information Security Program Plan, including customer governance, risk, compliance functions, and senior agency information security officer designation.</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -2139,12 +2139,12 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>RA-3</t>
+          <t>PM-9</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Risk Assessment</t>
+          <t>Risk Management Strategy</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Customer is responsible for conducting risk assessments of customer-deployed information systems at minimum annually and following any significant change, incorporating the AWS shared responsibility model and the customer-specific threat landscape.</t>
+          <t>Customer is responsible for developing and implementing the customer Risk Management Strategy, including risk tolerance levels for customer-managed workloads in AWS GovCloud and risk framing for the inherited and shared portions of the AWS shared responsibility model.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -2171,12 +2171,12 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>RA-5</t>
+          <t>RA-3</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Vulnerability Monitoring and Scanning</t>
+          <t>Risk Assessment</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -2186,12 +2186,12 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Not applicable to the AWS service boundary. AWS scans AWS-managed infrastructure independently per the AWS Vulnerability Management program.</t>
+          <t>Not applicable to the AWS service boundary.</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Customer is responsible for vulnerability scanning of customer-deployed workloads via Amazon Inspector (EC2, ECR, Lambda), customer third-party scanners (Tenable Nessus, Qualys, Rapid7), and remediating findings per customer-defined SLAs aligned to SI-2.</t>
+          <t>Customer is responsible for conducting risk assessments of customer-deployed information systems at minimum annually and following any significant change, incorporating the AWS shared responsibility model and the customer-specific threat landscape.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -2203,62 +2203,94 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>PE-10</t>
+          <t>RA-5</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Emergency Shutoff</t>
+          <t>Vulnerability Monitoring and Scanning</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>Customer</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Not applicable to AWS GovCloud (US) customer service offering. AWS datacenter emergency power shutoff is an AWS-internal facility control not exposed to customer interaction.</t>
+          <t>Not applicable to the AWS service boundary. AWS scans AWS-managed infrastructure independently per the AWS Vulnerability Management program.</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Not applicable to customer. Customer has no role in datacenter emergency shutoff procedures and no requirement to implement an equivalent compensating control.</t>
+          <t>Customer is responsible for vulnerability scanning of customer-deployed workloads via Amazon Inspector (EC2, ECR, Lambda), customer third-party scanners (Tenable Nessus, Qualys, Rapid7), and remediating findings per customer-defined SLAs aligned to SI-2.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Not Implemented</t>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
+          <t>PE-10</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Emergency Shutoff</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable to AWS GovCloud (US) customer service offering. AWS datacenter emergency power shutoff is an AWS-internal facility control not exposed to customer interaction.</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable to customer. Customer has no role in datacenter emergency shutoff procedures and no requirement to implement an equivalent compensating control.</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Not Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
           <t>PE-11</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>Emergency Power</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>Not Applicable</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>Not applicable to AWS GovCloud (US) customer service offering. AWS provides datacenter emergency power (UPS, generators, fuel reserves) as an internal infrastructure control.</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>Not applicable to customer. AWS GovCloud datacenter emergency power implementation is fully internal to AWS facilities; customer has no implementation or compensating-control responsibility.</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>Not Implemented</t>
         </is>

</xml_diff>